<commit_message>
refactored more create mv scripts
</commit_message>
<xml_diff>
--- a/cht_mv_ddls_old.xlsx
+++ b/cht_mv_ddls_old.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data Warehouse Work\CHT\community_health_datasets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{1B2BE85E-BE0B-4E74-85DF-CF1DA38304E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{9EEF5EEB-8ED6-486D-9B0E-17A1F394F940}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" xr2:uid="{13AD3CF5-9B19-4628-B9E1-A1C92EEF0F39}"/>
   </bookViews>
@@ -8363,7 +8363,7 @@
     <t>CRETE SIMILAR</t>
   </si>
   <si>
-    <t>REVISE QUERY</t>
+    <t>REVISE QUERY, rerun last</t>
   </si>
 </sst>
 </file>
@@ -10167,13 +10167,14 @@
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A57">
+      <c r="A57" s="3">
         <v>56</v>
       </c>
-      <c r="B57" t="s">
+      <c r="B57" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D57" t="s">
+      <c r="C57" s="3"/>
+      <c r="D57" s="3" t="s">
         <v>115</v>
       </c>
       <c r="E57" s="1" t="s">
@@ -10181,13 +10182,14 @@
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A58">
+      <c r="A58" s="3">
         <v>57</v>
       </c>
-      <c r="B58" t="s">
+      <c r="B58" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D58" t="s">
+      <c r="C58" s="3"/>
+      <c r="D58" s="3" t="s">
         <v>117</v>
       </c>
       <c r="E58" s="1" t="s">
@@ -10195,13 +10197,14 @@
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A59">
+      <c r="A59" s="3">
         <v>58</v>
       </c>
-      <c r="B59" t="s">
+      <c r="B59" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D59" t="s">
+      <c r="C59" s="3"/>
+      <c r="D59" s="3" t="s">
         <v>119</v>
       </c>
       <c r="E59" s="1" t="s">
@@ -10209,13 +10212,14 @@
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A60">
+      <c r="A60" s="4">
         <v>59</v>
       </c>
-      <c r="B60" t="s">
+      <c r="B60" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D60" t="s">
+      <c r="C60" s="4"/>
+      <c r="D60" s="4" t="s">
         <v>121</v>
       </c>
       <c r="E60" s="1" t="s">
@@ -10223,13 +10227,14 @@
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A61">
+      <c r="A61" s="3">
         <v>60</v>
       </c>
-      <c r="B61" t="s">
+      <c r="B61" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D61" t="s">
+      <c r="C61" s="3"/>
+      <c r="D61" s="3" t="s">
         <v>123</v>
       </c>
       <c r="E61" s="1" t="s">
@@ -10237,13 +10242,14 @@
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A62">
+      <c r="A62" s="3">
         <v>61</v>
       </c>
-      <c r="B62" t="s">
+      <c r="B62" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D62" t="s">
+      <c r="C62" s="3"/>
+      <c r="D62" s="3" t="s">
         <v>125</v>
       </c>
       <c r="E62" s="1" t="s">

</xml_diff>

<commit_message>
refactored more mv's by adding updated hierarchy
</commit_message>
<xml_diff>
--- a/cht_mv_ddls_old.xlsx
+++ b/cht_mv_ddls_old.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data Warehouse Work\CHT\community_health_datasets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{9EEF5EEB-8ED6-486D-9B0E-17A1F394F940}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFF6121F-0FBB-4343-AD6F-40BB01CF4CCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" xr2:uid="{13AD3CF5-9B19-4628-B9E1-A1C92EEF0F39}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="204">
   <si>
     <t>deps_id</t>
   </si>
@@ -7698,9 +7698,6 @@
   WHERE (((doc -&gt;&gt; 'form'::text) = 'training_evaluation'::text) AND is_current);</t>
   </si>
   <si>
-    <t>mv_treatment_follow_up_new</t>
-  </si>
-  <si>
     <t>CREATE MATERIALIZED VIEW cht.mv_treatment_follow_up_new AS  SELECT (doc -&gt;&gt; '_id'::text) AS doc_id,
     (doc -&gt;&gt; '_rev'::text) AS rev,
     to_timestamp((((NULLIF((doc -&gt;&gt; 'reported_date'::text), ''::text))::bigint / 1000))::double precision) AS reported,
@@ -8364,6 +8361,12 @@
   </si>
   <si>
     <t>REVISE QUERY, rerun last</t>
+  </si>
+  <si>
+    <t>CONFIRM HIERARCHY</t>
+  </si>
+  <si>
+    <t>mv_treatment_follow_up</t>
   </si>
 </sst>
 </file>
@@ -9262,14 +9265,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87D4D036-6DF8-400A-9DA7-59F70A962B06}">
-  <dimension ref="A1:F94"/>
+  <dimension ref="A1:F95"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14.08984375" customWidth="1"/>
     <col min="2" max="3" width="14.36328125" customWidth="1"/>
     <col min="4" max="4" width="43.453125" customWidth="1"/>
     <col min="5" max="5" width="27.08984375" customWidth="1"/>
-    <col min="6" max="6" width="17.7265625" customWidth="1"/>
+    <col min="6" max="6" width="19.7265625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
@@ -9280,7 +9283,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>2</v>
@@ -9289,7 +9292,7 @@
         <v>3</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
@@ -9359,7 +9362,7 @@
         <v>4</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>13</v>
@@ -9391,7 +9394,7 @@
         <v>4</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D8" s="4" t="s">
         <v>17</v>
@@ -9438,7 +9441,7 @@
         <v>4</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D11" s="4" t="s">
         <v>23</v>
@@ -9545,7 +9548,7 @@
         <v>4</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D18" s="5" t="s">
         <v>37</v>
@@ -9554,7 +9557,7 @@
         <v>38</v>
       </c>
       <c r="F18" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.35">
@@ -9565,7 +9568,7 @@
         <v>4</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D19" s="6" t="s">
         <v>39</v>
@@ -9600,7 +9603,7 @@
         <v>4</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D21" s="4" t="s">
         <v>43</v>
@@ -9609,7 +9612,7 @@
         <v>44</v>
       </c>
       <c r="F21" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.35">
@@ -9650,7 +9653,7 @@
         <v>4</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D24" s="4" t="s">
         <v>49</v>
@@ -9727,7 +9730,7 @@
         <v>4</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D29" s="6" t="s">
         <v>59</v>
@@ -9744,7 +9747,7 @@
         <v>4</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D30" s="6" t="s">
         <v>61</v>
@@ -9776,7 +9779,7 @@
         <v>4</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="D32" s="6" t="s">
         <v>65</v>
@@ -9785,7 +9788,7 @@
         <v>66</v>
       </c>
       <c r="F32" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.35">
@@ -9811,7 +9814,7 @@
         <v>4</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D34" s="4" t="s">
         <v>69</v>
@@ -9843,7 +9846,7 @@
         <v>4</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D36" s="6" t="s">
         <v>73</v>
@@ -9875,7 +9878,7 @@
         <v>4</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D38" s="6" t="s">
         <v>77</v>
@@ -9907,7 +9910,7 @@
         <v>4</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D40" s="4" t="s">
         <v>81</v>
@@ -9939,7 +9942,7 @@
         <v>4</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="D42" s="6" t="s">
         <v>85</v>
@@ -10121,7 +10124,7 @@
         <v>4</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D54" s="4" t="s">
         <v>109</v>
@@ -10130,7 +10133,7 @@
         <v>110</v>
       </c>
       <c r="F54" s="4" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.35">
@@ -10148,7 +10151,7 @@
         <v>112</v>
       </c>
       <c r="F55" s="6" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.35">
@@ -10257,13 +10260,14 @@
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A63">
+      <c r="A63" s="3">
         <v>62</v>
       </c>
-      <c r="B63" t="s">
+      <c r="B63" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D63" t="s">
+      <c r="C63" s="3"/>
+      <c r="D63" s="3" t="s">
         <v>127</v>
       </c>
       <c r="E63" s="1" t="s">
@@ -10271,251 +10275,280 @@
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A64">
+      <c r="A64" s="3">
         <v>63</v>
       </c>
-      <c r="B64" t="s">
+      <c r="B64" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D64" t="s">
+      <c r="C64" s="3"/>
+      <c r="D64" s="3" t="s">
         <v>129</v>
       </c>
       <c r="E64" s="1" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A65">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A65" s="3">
         <v>64</v>
       </c>
-      <c r="B65" t="s">
+      <c r="B65" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D65" t="s">
+      <c r="C65" s="3"/>
+      <c r="D65" s="3" t="s">
         <v>131</v>
       </c>
       <c r="E65" s="1" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A66">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A66" s="6">
         <v>65</v>
       </c>
-      <c r="B66" t="s">
+      <c r="B66" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="D66" t="s">
+      <c r="C66" s="6" t="s">
+        <v>199</v>
+      </c>
+      <c r="D66" s="6" t="s">
         <v>133</v>
       </c>
       <c r="E66" s="1" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A67">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A67" s="6">
         <v>66</v>
       </c>
-      <c r="B67" t="s">
+      <c r="B67" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="D67" t="s">
+      <c r="C67" s="6"/>
+      <c r="D67" s="6" t="s">
         <v>135</v>
       </c>
       <c r="E67" s="1" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A68">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A68" s="4">
         <v>67</v>
       </c>
-      <c r="B68" t="s">
+      <c r="B68" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D68" t="s">
+      <c r="C68" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="D68" s="4" t="s">
         <v>137</v>
       </c>
       <c r="E68" s="1" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A69">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A69" s="4">
         <v>68</v>
       </c>
-      <c r="B69" t="s">
+      <c r="B69" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D69" t="s">
+      <c r="C69" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="D69" s="4" t="s">
         <v>139</v>
       </c>
       <c r="E69" s="1" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A70">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A70" s="4">
         <v>69</v>
       </c>
-      <c r="B70" t="s">
+      <c r="B70" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D70" t="s">
+      <c r="C70" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="D70" s="4" t="s">
         <v>141</v>
       </c>
       <c r="E70" s="1" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A71">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A71" s="3">
         <v>70</v>
       </c>
-      <c r="B71" t="s">
+      <c r="B71" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D71" t="s">
+      <c r="C71" s="3"/>
+      <c r="D71" s="3" t="s">
         <v>143</v>
       </c>
       <c r="E71" s="1" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A72">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A72" s="3">
         <v>71</v>
       </c>
-      <c r="B72" t="s">
+      <c r="B72" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D72" t="s">
+      <c r="C72" s="3"/>
+      <c r="D72" s="3" t="s">
         <v>145</v>
       </c>
       <c r="E72" s="1" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A73">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A73" s="3">
         <v>72</v>
       </c>
-      <c r="B73" t="s">
+      <c r="B73" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D73" t="s">
+      <c r="C73" s="3"/>
+      <c r="D73" s="3" t="s">
         <v>147</v>
       </c>
       <c r="E73" s="1" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A74">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A74" s="3">
         <v>73</v>
       </c>
-      <c r="B74" t="s">
+      <c r="B74" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D74" t="s">
+      <c r="C74" s="3"/>
+      <c r="D74" s="3" t="s">
         <v>149</v>
       </c>
       <c r="E74" s="1" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A75">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A75" s="3">
         <v>74</v>
       </c>
-      <c r="B75" t="s">
+      <c r="B75" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D75" t="s">
+      <c r="C75" s="3"/>
+      <c r="D75" s="3" t="s">
         <v>151</v>
       </c>
       <c r="E75" s="1" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A76">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A76" s="3">
         <v>75</v>
       </c>
-      <c r="B76" t="s">
+      <c r="B76" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D76" t="s">
+      <c r="C76" s="3"/>
+      <c r="D76" s="3" t="s">
         <v>153</v>
       </c>
       <c r="E76" s="1" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A77">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A77" s="3">
         <v>76</v>
       </c>
-      <c r="B77" t="s">
+      <c r="B77" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D77" t="s">
+      <c r="C77" s="3"/>
+      <c r="D77" s="3" t="s">
         <v>155</v>
       </c>
       <c r="E77" s="1" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A78">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A78" s="3">
         <v>77</v>
       </c>
-      <c r="B78" t="s">
+      <c r="B78" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D78" t="s">
+      <c r="C78" s="3"/>
+      <c r="D78" s="3" t="s">
         <v>157</v>
       </c>
       <c r="E78" s="1" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A79">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A79" s="3">
         <v>78</v>
       </c>
-      <c r="B79" t="s">
+      <c r="B79" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D79" t="s">
+      <c r="C79" s="3"/>
+      <c r="D79" s="3" t="s">
         <v>159</v>
       </c>
       <c r="E79" s="1" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A80">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A80" s="6">
         <v>79</v>
       </c>
-      <c r="B80" t="s">
+      <c r="B80" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="D80" t="s">
+      <c r="C80" s="6"/>
+      <c r="D80" s="6" t="s">
         <v>161</v>
       </c>
       <c r="E80" s="1" t="s">
         <v>162</v>
       </c>
+      <c r="F80" s="6" t="s">
+        <v>202</v>
+      </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A81">
+      <c r="A81" s="3">
         <v>80</v>
       </c>
-      <c r="B81" t="s">
+      <c r="B81" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D81" t="s">
+      <c r="C81" s="3"/>
+      <c r="D81" s="3" t="s">
         <v>163</v>
       </c>
       <c r="E81" s="1" t="s">
@@ -10523,13 +10556,14 @@
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A82">
+      <c r="A82" s="3">
         <v>81</v>
       </c>
-      <c r="B82" t="s">
+      <c r="B82" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D82" t="s">
+      <c r="C82" s="3"/>
+      <c r="D82" s="3" t="s">
         <v>165</v>
       </c>
       <c r="E82" s="1" t="s">
@@ -10537,13 +10571,14 @@
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A83">
+      <c r="A83" s="3">
         <v>82</v>
       </c>
-      <c r="B83" t="s">
+      <c r="B83" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D83" t="s">
+      <c r="C83" s="3"/>
+      <c r="D83" s="3" t="s">
         <v>167</v>
       </c>
       <c r="E83" s="1" t="s">
@@ -10551,13 +10586,14 @@
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A84">
+      <c r="A84" s="3">
         <v>83</v>
       </c>
-      <c r="B84" t="s">
+      <c r="B84" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D84" t="s">
+      <c r="C84" s="3"/>
+      <c r="D84" s="3" t="s">
         <v>169</v>
       </c>
       <c r="E84" s="1" t="s">
@@ -10565,13 +10601,14 @@
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A85">
+      <c r="A85" s="3">
         <v>84</v>
       </c>
-      <c r="B85" t="s">
+      <c r="B85" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D85" t="s">
+      <c r="C85" s="3"/>
+      <c r="D85" s="3" t="s">
         <v>171</v>
       </c>
       <c r="E85" s="1" t="s">
@@ -10579,59 +10616,63 @@
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A86">
+      <c r="A86" s="3">
         <v>85</v>
       </c>
-      <c r="B86" t="s">
+      <c r="B86" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D86" t="s">
+      <c r="C86" s="3"/>
+      <c r="D86" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="E86" s="1" t="s">
         <v>173</v>
-      </c>
-      <c r="E86" s="1" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A87">
+      <c r="A87" s="3">
         <v>86</v>
       </c>
-      <c r="B87" t="s">
+      <c r="B87" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D87" t="s">
+      <c r="C87" s="3"/>
+      <c r="D87" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E87" s="1" t="s">
         <v>175</v>
-      </c>
-      <c r="E87" s="1" t="s">
-        <v>176</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A88">
+      <c r="A88" s="3">
         <v>87</v>
       </c>
-      <c r="B88" t="s">
+      <c r="B88" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D88" t="s">
+      <c r="C88" s="3"/>
+      <c r="D88" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="E88" s="1" t="s">
         <v>177</v>
-      </c>
-      <c r="E88" s="1" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A89">
+      <c r="A89" s="3">
         <v>88</v>
       </c>
-      <c r="B89" t="s">
+      <c r="B89" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D89" t="s">
+      <c r="C89" s="3"/>
+      <c r="D89" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="E89" s="1" t="s">
         <v>179</v>
-      </c>
-      <c r="E89" s="1" t="s">
-        <v>180</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.35">
@@ -10642,10 +10683,10 @@
         <v>4</v>
       </c>
       <c r="D90" t="s">
+        <v>180</v>
+      </c>
+      <c r="E90" s="1" t="s">
         <v>181</v>
-      </c>
-      <c r="E90" s="1" t="s">
-        <v>182</v>
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.35">
@@ -10656,10 +10697,10 @@
         <v>4</v>
       </c>
       <c r="D91" t="s">
+        <v>182</v>
+      </c>
+      <c r="E91" s="1" t="s">
         <v>183</v>
-      </c>
-      <c r="E91" s="1" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.35">
@@ -10670,10 +10711,10 @@
         <v>4</v>
       </c>
       <c r="D92" t="s">
+        <v>184</v>
+      </c>
+      <c r="E92" s="1" t="s">
         <v>185</v>
-      </c>
-      <c r="E92" s="1" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.35">
@@ -10684,10 +10725,10 @@
         <v>4</v>
       </c>
       <c r="D93" t="s">
+        <v>186</v>
+      </c>
+      <c r="E93" s="1" t="s">
         <v>187</v>
-      </c>
-      <c r="E93" s="1" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.35">
@@ -10698,11 +10739,14 @@
         <v>4</v>
       </c>
       <c r="D94" t="s">
+        <v>188</v>
+      </c>
+      <c r="E94" s="1" t="s">
         <v>189</v>
       </c>
-      <c r="E94" s="1" t="s">
-        <v>190</v>
-      </c>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E95" s="1"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:F1" xr:uid="{87D4D036-6DF8-400A-9DA7-59F70A962B06}"/>

</xml_diff>

<commit_message>
added script for creating tables on devtest server
</commit_message>
<xml_diff>
--- a/cht_mv_ddls_old.xlsx
+++ b/cht_mv_ddls_old.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data Warehouse Work\CHT\community_health_datasets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFF6121F-0FBB-4343-AD6F-40BB01CF4CCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53B668D0-4E61-47B9-8D94-D73FB598464A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" xr2:uid="{13AD3CF5-9B19-4628-B9E1-A1C92EEF0F39}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="204">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="207">
   <si>
     <t>deps_id</t>
   </si>
@@ -8368,6 +8368,15 @@
   <si>
     <t>mv_treatment_follow_up</t>
   </si>
+  <si>
+    <t>REVISE QUERY</t>
+  </si>
+  <si>
+    <t>check xml for corect columns (looks like some were left out)</t>
+  </si>
+  <si>
+    <t>non existent</t>
+  </si>
 </sst>
 </file>
 
@@ -8509,7 +8518,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="38">
+  <fills count="37">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -8709,12 +8718,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -8880,7 +8883,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -8889,7 +8892,6 @@
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -9355,20 +9357,23 @@
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A6" s="4">
+      <c r="A6" s="5">
         <v>5</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="5" t="s">
         <v>191</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>14</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
@@ -9387,16 +9392,16 @@
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A8" s="4">
+      <c r="A8" s="3">
         <v>7</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="3" t="s">
         <v>191</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E8" s="1" t="s">
@@ -9404,14 +9409,14 @@
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A9" s="4">
+      <c r="A9" s="3">
         <v>8</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4" t="s">
+      <c r="C9" s="3"/>
+      <c r="D9" s="3" t="s">
         <v>19</v>
       </c>
       <c r="E9" s="1" t="s">
@@ -9451,14 +9456,14 @@
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A12" s="4">
+      <c r="A12" s="3">
         <v>11</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4" t="s">
+      <c r="C12" s="3"/>
+      <c r="D12" s="3" t="s">
         <v>25</v>
       </c>
       <c r="E12" s="1" t="s">
@@ -9466,14 +9471,14 @@
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A13" s="4">
+      <c r="A13" s="3">
         <v>12</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C13" s="4"/>
-      <c r="D13" s="4" t="s">
+      <c r="C13" s="3"/>
+      <c r="D13" s="3" t="s">
         <v>27</v>
       </c>
       <c r="E13" s="1" t="s">
@@ -9561,16 +9566,16 @@
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A19" s="6">
+      <c r="A19" s="5">
         <v>18</v>
       </c>
-      <c r="B19" s="6" t="s">
+      <c r="B19" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="C19" s="5" t="s">
         <v>192</v>
       </c>
-      <c r="D19" s="6" t="s">
+      <c r="D19" s="5" t="s">
         <v>39</v>
       </c>
       <c r="E19" s="1" t="s">
@@ -9646,16 +9651,16 @@
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A24" s="4">
+      <c r="A24" s="3">
         <v>23</v>
       </c>
-      <c r="B24" s="4" t="s">
+      <c r="B24" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C24" s="4" t="s">
+      <c r="C24" s="3" t="s">
         <v>191</v>
       </c>
-      <c r="D24" s="4" t="s">
+      <c r="D24" s="3" t="s">
         <v>49</v>
       </c>
       <c r="E24" s="1" t="s">
@@ -9663,14 +9668,14 @@
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A25" s="4">
+      <c r="A25" s="3">
         <v>24</v>
       </c>
-      <c r="B25" s="4" t="s">
+      <c r="B25" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C25" s="4"/>
-      <c r="D25" s="4" t="s">
+      <c r="C25" s="3"/>
+      <c r="D25" s="3" t="s">
         <v>51</v>
       </c>
       <c r="E25" s="1" t="s">
@@ -9678,14 +9683,14 @@
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A26" s="4">
+      <c r="A26" s="3">
         <v>25</v>
       </c>
-      <c r="B26" s="4" t="s">
+      <c r="B26" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C26" s="4"/>
-      <c r="D26" s="4" t="s">
+      <c r="C26" s="3"/>
+      <c r="D26" s="3" t="s">
         <v>53</v>
       </c>
       <c r="E26" s="1" t="s">
@@ -9723,16 +9728,16 @@
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A29" s="6">
+      <c r="A29" s="5">
         <v>28</v>
       </c>
-      <c r="B29" s="6" t="s">
+      <c r="B29" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C29" s="6" t="s">
+      <c r="C29" s="5" t="s">
         <v>192</v>
       </c>
-      <c r="D29" s="6" t="s">
+      <c r="D29" s="5" t="s">
         <v>59</v>
       </c>
       <c r="E29" s="1" t="s">
@@ -9740,16 +9745,16 @@
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A30" s="6">
+      <c r="A30" s="5">
         <v>29</v>
       </c>
-      <c r="B30" s="6" t="s">
+      <c r="B30" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C30" s="6" t="s">
+      <c r="C30" s="5" t="s">
         <v>192</v>
       </c>
-      <c r="D30" s="6" t="s">
+      <c r="D30" s="5" t="s">
         <v>61</v>
       </c>
       <c r="E30" s="1" t="s">
@@ -9757,14 +9762,14 @@
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A31" s="4">
+      <c r="A31" s="3">
         <v>30</v>
       </c>
-      <c r="B31" s="4" t="s">
+      <c r="B31" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C31" s="4"/>
-      <c r="D31" s="4" t="s">
+      <c r="C31" s="3"/>
+      <c r="D31" s="3" t="s">
         <v>63</v>
       </c>
       <c r="E31" s="1" t="s">
@@ -9772,16 +9777,16 @@
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A32" s="6">
+      <c r="A32" s="5">
         <v>31</v>
       </c>
-      <c r="B32" s="6" t="s">
+      <c r="B32" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C32" s="6" t="s">
+      <c r="C32" s="5" t="s">
         <v>196</v>
       </c>
-      <c r="D32" s="6" t="s">
+      <c r="D32" s="5" t="s">
         <v>65</v>
       </c>
       <c r="E32" s="1" t="s">
@@ -9791,7 +9796,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A33" s="3">
         <v>32</v>
       </c>
@@ -9805,57 +9810,60 @@
       <c r="E33" s="1" t="s">
         <v>68</v>
       </c>
+      <c r="F33" s="3" t="s">
+        <v>205</v>
+      </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A34" s="4">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A34" s="3">
         <v>33</v>
       </c>
-      <c r="B34" s="4" t="s">
+      <c r="B34" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C34" s="4" t="s">
+      <c r="C34" s="3" t="s">
         <v>191</v>
       </c>
-      <c r="D34" s="4" t="s">
+      <c r="D34" s="3" t="s">
         <v>69</v>
       </c>
       <c r="E34" s="1" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A35" s="4">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A35" s="3">
         <v>34</v>
       </c>
-      <c r="B35" s="4" t="s">
+      <c r="B35" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C35" s="4"/>
-      <c r="D35" s="4" t="s">
+      <c r="C35" s="3"/>
+      <c r="D35" s="3" t="s">
         <v>71</v>
       </c>
       <c r="E35" s="1" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A36" s="6">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A36" s="3">
         <v>35</v>
       </c>
-      <c r="B36" s="6" t="s">
+      <c r="B36" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C36" s="6" t="s">
+      <c r="C36" s="3" t="s">
         <v>198</v>
       </c>
-      <c r="D36" s="6" t="s">
+      <c r="D36" s="3" t="s">
         <v>73</v>
       </c>
       <c r="E36" s="1" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A37" s="3">
         <v>36</v>
       </c>
@@ -9870,24 +9878,24 @@
         <v>76</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A38" s="6">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A38" s="3">
         <v>37</v>
       </c>
-      <c r="B38" s="6" t="s">
+      <c r="B38" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C38" s="6" t="s">
+      <c r="C38" s="3" t="s">
         <v>198</v>
       </c>
-      <c r="D38" s="6" t="s">
+      <c r="D38" s="3" t="s">
         <v>77</v>
       </c>
       <c r="E38" s="1" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A39" s="3">
         <v>38</v>
       </c>
@@ -9902,7 +9910,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A40" s="4">
         <v>39</v>
       </c>
@@ -9919,7 +9927,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A41" s="3">
         <v>40</v>
       </c>
@@ -9934,24 +9942,24 @@
         <v>84</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A42" s="6">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A42" s="5">
         <v>41</v>
       </c>
-      <c r="B42" s="6" t="s">
+      <c r="B42" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C42" s="6" t="s">
+      <c r="C42" s="5" t="s">
         <v>199</v>
       </c>
-      <c r="D42" s="6" t="s">
+      <c r="D42" s="5" t="s">
         <v>85</v>
       </c>
       <c r="E42" s="1" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A43" s="3">
         <v>42</v>
       </c>
@@ -9966,7 +9974,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A44" s="3">
         <v>43</v>
       </c>
@@ -9981,7 +9989,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A45" s="3">
         <v>44</v>
       </c>
@@ -9996,45 +10004,45 @@
         <v>92</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A46" s="4">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A46" s="3">
         <v>45</v>
       </c>
-      <c r="B46" s="4" t="s">
+      <c r="B46" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C46" s="4"/>
-      <c r="D46" s="4" t="s">
+      <c r="C46" s="3"/>
+      <c r="D46" s="3" t="s">
         <v>93</v>
       </c>
       <c r="E46" s="1" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A47" s="4">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A47" s="3">
         <v>46</v>
       </c>
-      <c r="B47" s="4" t="s">
+      <c r="B47" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C47" s="4"/>
-      <c r="D47" s="4" t="s">
+      <c r="C47" s="3"/>
+      <c r="D47" s="3" t="s">
         <v>95</v>
       </c>
       <c r="E47" s="1" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A48" s="4">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A48" s="3">
         <v>47</v>
       </c>
-      <c r="B48" s="4" t="s">
+      <c r="B48" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C48" s="4"/>
-      <c r="D48" s="4" t="s">
+      <c r="C48" s="3"/>
+      <c r="D48" s="3" t="s">
         <v>97</v>
       </c>
       <c r="E48" s="1" t="s">
@@ -10042,14 +10050,14 @@
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A49" s="4">
+      <c r="A49" s="3">
         <v>48</v>
       </c>
-      <c r="B49" s="4" t="s">
+      <c r="B49" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C49" s="4"/>
-      <c r="D49" s="4" t="s">
+      <c r="C49" s="3"/>
+      <c r="D49" s="3" t="s">
         <v>99</v>
       </c>
       <c r="E49" s="1" t="s">
@@ -10057,14 +10065,14 @@
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A50" s="4">
+      <c r="A50" s="3">
         <v>49</v>
       </c>
-      <c r="B50" s="4" t="s">
+      <c r="B50" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C50" s="4"/>
-      <c r="D50" s="4" t="s">
+      <c r="C50" s="3"/>
+      <c r="D50" s="3" t="s">
         <v>101</v>
       </c>
       <c r="E50" s="1" t="s">
@@ -10072,14 +10080,14 @@
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A51" s="4">
+      <c r="A51" s="3">
         <v>50</v>
       </c>
-      <c r="B51" s="4" t="s">
+      <c r="B51" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C51" s="4"/>
-      <c r="D51" s="4" t="s">
+      <c r="C51" s="3"/>
+      <c r="D51" s="3" t="s">
         <v>103</v>
       </c>
       <c r="E51" s="1" t="s">
@@ -10087,14 +10095,14 @@
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A52" s="4">
+      <c r="A52" s="3">
         <v>51</v>
       </c>
-      <c r="B52" s="4" t="s">
+      <c r="B52" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C52" s="4"/>
-      <c r="D52" s="4" t="s">
+      <c r="C52" s="3"/>
+      <c r="D52" s="3" t="s">
         <v>105</v>
       </c>
       <c r="E52" s="1" t="s">
@@ -10137,32 +10145,32 @@
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A55" s="6">
+      <c r="A55" s="5">
         <v>54</v>
       </c>
-      <c r="B55" s="6" t="s">
+      <c r="B55" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C55" s="6"/>
-      <c r="D55" s="6" t="s">
+      <c r="C55" s="5"/>
+      <c r="D55" s="5" t="s">
         <v>111</v>
       </c>
       <c r="E55" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="F55" s="6" t="s">
+      <c r="F55" s="5" t="s">
         <v>201</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A56" s="4">
+      <c r="A56" s="3">
         <v>55</v>
       </c>
-      <c r="B56" s="4" t="s">
+      <c r="B56" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C56" s="4"/>
-      <c r="D56" s="4" t="s">
+      <c r="C56" s="3"/>
+      <c r="D56" s="3" t="s">
         <v>113</v>
       </c>
       <c r="E56" s="1" t="s">
@@ -10305,16 +10313,16 @@
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A66" s="6">
+      <c r="A66" s="5">
         <v>65</v>
       </c>
-      <c r="B66" s="6" t="s">
+      <c r="B66" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C66" s="6" t="s">
+      <c r="C66" s="5" t="s">
         <v>199</v>
       </c>
-      <c r="D66" s="6" t="s">
+      <c r="D66" s="5" t="s">
         <v>133</v>
       </c>
       <c r="E66" s="1" t="s">
@@ -10322,14 +10330,16 @@
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A67" s="6">
+      <c r="A67" s="5">
         <v>66</v>
       </c>
-      <c r="B67" s="6" t="s">
+      <c r="B67" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C67" s="6"/>
-      <c r="D67" s="6" t="s">
+      <c r="C67" s="5" t="s">
+        <v>199</v>
+      </c>
+      <c r="D67" s="5" t="s">
         <v>135</v>
       </c>
       <c r="E67" s="1" t="s">
@@ -10337,16 +10347,16 @@
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A68" s="4">
+      <c r="A68" s="3">
         <v>67</v>
       </c>
-      <c r="B68" s="4" t="s">
+      <c r="B68" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C68" s="4" t="s">
+      <c r="C68" s="3" t="s">
         <v>191</v>
       </c>
-      <c r="D68" s="4" t="s">
+      <c r="D68" s="3" t="s">
         <v>137</v>
       </c>
       <c r="E68" s="1" t="s">
@@ -10354,16 +10364,16 @@
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A69" s="4">
+      <c r="A69" s="3">
         <v>68</v>
       </c>
-      <c r="B69" s="4" t="s">
+      <c r="B69" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C69" s="4" t="s">
+      <c r="C69" s="3" t="s">
         <v>191</v>
       </c>
-      <c r="D69" s="4" t="s">
+      <c r="D69" s="3" t="s">
         <v>139</v>
       </c>
       <c r="E69" s="1" t="s">
@@ -10371,16 +10381,16 @@
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A70" s="4">
+      <c r="A70" s="3">
         <v>69</v>
       </c>
-      <c r="B70" s="4" t="s">
+      <c r="B70" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C70" s="4" t="s">
+      <c r="C70" s="3" t="s">
         <v>191</v>
       </c>
-      <c r="D70" s="4" t="s">
+      <c r="D70" s="3" t="s">
         <v>141</v>
       </c>
       <c r="E70" s="1" t="s">
@@ -10523,24 +10533,24 @@
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A80" s="6">
+      <c r="A80" s="5">
         <v>79</v>
       </c>
-      <c r="B80" s="6" t="s">
+      <c r="B80" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C80" s="6"/>
-      <c r="D80" s="6" t="s">
+      <c r="C80" s="5"/>
+      <c r="D80" s="5" t="s">
         <v>161</v>
       </c>
       <c r="E80" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="F80" s="6" t="s">
+      <c r="F80" s="5" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A81" s="3">
         <v>80</v>
       </c>
@@ -10555,7 +10565,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A82" s="3">
         <v>81</v>
       </c>
@@ -10570,7 +10580,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A83" s="3">
         <v>82</v>
       </c>
@@ -10585,7 +10595,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A84" s="3">
         <v>83</v>
       </c>
@@ -10600,7 +10610,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A85" s="3">
         <v>84</v>
       </c>
@@ -10615,7 +10625,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A86" s="3">
         <v>85</v>
       </c>
@@ -10630,7 +10640,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A87" s="3">
         <v>86</v>
       </c>
@@ -10645,7 +10655,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A88" s="3">
         <v>87</v>
       </c>
@@ -10660,7 +10670,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A89" s="3">
         <v>88</v>
       </c>
@@ -10675,63 +10685,74 @@
         <v>179</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A90">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A90" s="5">
         <v>89</v>
       </c>
-      <c r="B90" t="s">
+      <c r="B90" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D90" t="s">
+      <c r="C90" s="5" t="s">
+        <v>199</v>
+      </c>
+      <c r="D90" s="5" t="s">
         <v>180</v>
       </c>
       <c r="E90" s="1" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A91">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A91" s="5">
         <v>90</v>
       </c>
-      <c r="B91" t="s">
+      <c r="B91" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D91" t="s">
+      <c r="C91" s="5"/>
+      <c r="D91" s="5" t="s">
         <v>182</v>
       </c>
       <c r="E91" s="1" t="s">
         <v>183</v>
       </c>
+      <c r="F91" s="5" t="s">
+        <v>204</v>
+      </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A92">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A92" s="5">
         <v>91</v>
       </c>
-      <c r="B92" t="s">
+      <c r="B92" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D92" t="s">
+      <c r="C92" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="D92" s="5" t="s">
         <v>184</v>
       </c>
       <c r="E92" s="1" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A93">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A93" s="3">
         <v>92</v>
       </c>
-      <c r="B93" t="s">
+      <c r="B93" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D93" t="s">
+      <c r="C93" s="3"/>
+      <c r="D93" s="3" t="s">
         <v>186</v>
       </c>
       <c r="E93" s="1" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A94">
         <v>93</v>
       </c>
@@ -10745,7 +10766,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.35">
       <c r="E95" s="1"/>
     </row>
   </sheetData>

</xml_diff>